<commit_message>
Made the default frequency range and the persistent frequency range for the brace separate from the other types. The persistent is different for each type (classical, acoustic, flamenco, plate, brace).
</commit_message>
<xml_diff>
--- a/Wood Property Measurementsl.xlsx
+++ b/Wood Property Measurementsl.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dws/Library/CloudStorage/Dropbox/Programming/src/GuitarTap/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dws/src/GuitarTap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3CF8BFB-D467-C743-8170-7D156DCC6726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A0A16AF-5484-7B44-8F99-5E13CF50A3E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2100" yWindow="2540" windowWidth="30240" windowHeight="16640" tabRatio="768" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1880" windowWidth="30240" windowHeight="16640" tabRatio="768" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monopole Mobility" sheetId="10" r:id="rId1"/>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="265">
   <si>
     <t>E</t>
   </si>
@@ -1518,10 +1518,16 @@
     <t>Flexural Rigidity</t>
   </si>
   <si>
-    <t>Spruce</t>
-  </si>
-  <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Spruce (mac)</t>
+  </si>
+  <si>
+    <t>Spruce (ipad)</t>
+  </si>
+  <si>
+    <t>Spruce (iphone)</t>
   </si>
 </sst>
 </file>
@@ -2283,7 +2289,7 @@
       <alignment horizontal="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="278">
+  <cellXfs count="279">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -2916,6 +2922,15 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -2926,15 +2941,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2960,6 +2966,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3936,8 +3945,8 @@
       <xdr:row>15</xdr:row>
       <xdr:rowOff>102774</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="TextBox 2">
@@ -4190,7 +4199,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="TextBox 2">
@@ -4329,8 +4338,8 @@
       <xdr:row>19</xdr:row>
       <xdr:rowOff>136600</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="TextBox 3">
@@ -4656,7 +4665,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="TextBox 3">
@@ -15700,7 +15709,7 @@
   <sheetPr codeName="Sheet4">
     <tabColor indexed="27"/>
   </sheetPr>
-  <dimension ref="A1:Q41"/>
+  <dimension ref="A1:Q43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="3" max="3" width="10.33203125" customWidth="1"/>
@@ -15823,7 +15832,7 @@
       </c>
       <c r="K12" s="4"/>
       <c r="N12" s="258" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="Q12" s="258">
         <f>Q11*Q11/SQRT(48*PI()*PI())</f>
@@ -16278,8 +16287,8 @@
       <c r="L40" s="40"/>
     </row>
     <row r="41" spans="4:12" x14ac:dyDescent="0.15">
-      <c r="D41" s="71" t="s">
-        <v>261</v>
+      <c r="D41" s="278" t="s">
+        <v>262</v>
       </c>
       <c r="E41">
         <v>512.1</v>
@@ -16301,8 +16310,64 @@
         <v>384.87782781015801</v>
       </c>
       <c r="L41">
-        <f>((E12*F12^2)/(1.0279*G12))^2*J12/1000000000</f>
+        <f>((E41*F41^2)/(1.0279*G41))^2*J41/1000000000</f>
         <v>10.597749931493331</v>
+      </c>
+    </row>
+    <row r="42" spans="4:12" x14ac:dyDescent="0.15">
+      <c r="D42" s="278" t="s">
+        <v>263</v>
+      </c>
+      <c r="E42">
+        <v>512.70000000000005</v>
+      </c>
+      <c r="F42">
+        <v>0.55600000000000005</v>
+      </c>
+      <c r="G42">
+        <v>2.9350000000000001E-2</v>
+      </c>
+      <c r="H42">
+        <v>2.0379999999999999E-2</v>
+      </c>
+      <c r="I42">
+        <v>0.128</v>
+      </c>
+      <c r="J42">
+        <f>I42/(H42*G42*F42)</f>
+        <v>384.87782781015801</v>
+      </c>
+      <c r="L42">
+        <f>((E42*F42^2)/(1.0279*G42))^2*J42/1000000000</f>
+        <v>10.622598105689029</v>
+      </c>
+    </row>
+    <row r="43" spans="4:12" x14ac:dyDescent="0.15">
+      <c r="D43" s="278" t="s">
+        <v>264</v>
+      </c>
+      <c r="E43">
+        <v>512</v>
+      </c>
+      <c r="F43">
+        <v>0.55600000000000005</v>
+      </c>
+      <c r="G43">
+        <v>2.9350000000000001E-2</v>
+      </c>
+      <c r="H43">
+        <v>2.0379999999999999E-2</v>
+      </c>
+      <c r="I43">
+        <v>0.128</v>
+      </c>
+      <c r="J43">
+        <f>I43/(H43*G43*F43)</f>
+        <v>384.87782781015801</v>
+      </c>
+      <c r="L43">
+        <f>((E43*F43^2)/(1.0279*G43))^2*J43/1000000000</f>
+        <v>10.593611397926807</v>
       </c>
     </row>
   </sheetData>
@@ -17181,64 +17246,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.15">
-      <c r="A1" s="267" t="s">
+      <c r="A1" s="263" t="s">
         <v>195</v>
       </c>
-      <c r="B1" s="267"/>
-      <c r="C1" s="267"/>
-      <c r="D1" s="267"/>
-      <c r="E1" s="267"/>
-      <c r="F1" s="267"/>
-      <c r="G1" s="267"/>
-      <c r="H1" s="267"/>
-      <c r="I1" s="267"/>
-      <c r="J1" s="267"/>
-      <c r="K1" s="267"/>
-      <c r="L1" s="267"/>
-      <c r="M1" s="267"/>
-      <c r="N1" s="267"/>
-      <c r="O1" s="267"/>
-      <c r="P1" s="267"/>
-      <c r="Q1" s="267"/>
-      <c r="R1" s="267"/>
-      <c r="S1" s="267"/>
-      <c r="T1" s="267"/>
-      <c r="U1" s="267"/>
-      <c r="V1" s="267"/>
-      <c r="W1" s="267"/>
-      <c r="X1" s="267"/>
-      <c r="Y1" s="267"/>
-      <c r="Z1" s="267"/>
+      <c r="B1" s="263"/>
+      <c r="C1" s="263"/>
+      <c r="D1" s="263"/>
+      <c r="E1" s="263"/>
+      <c r="F1" s="263"/>
+      <c r="G1" s="263"/>
+      <c r="H1" s="263"/>
+      <c r="I1" s="263"/>
+      <c r="J1" s="263"/>
+      <c r="K1" s="263"/>
+      <c r="L1" s="263"/>
+      <c r="M1" s="263"/>
+      <c r="N1" s="263"/>
+      <c r="O1" s="263"/>
+      <c r="P1" s="263"/>
+      <c r="Q1" s="263"/>
+      <c r="R1" s="263"/>
+      <c r="S1" s="263"/>
+      <c r="T1" s="263"/>
+      <c r="U1" s="263"/>
+      <c r="V1" s="263"/>
+      <c r="W1" s="263"/>
+      <c r="X1" s="263"/>
+      <c r="Y1" s="263"/>
+      <c r="Z1" s="263"/>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.15">
-      <c r="A2" s="267" t="s">
+      <c r="A2" s="263" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="267"/>
-      <c r="C2" s="267"/>
-      <c r="D2" s="267"/>
-      <c r="E2" s="267"/>
-      <c r="F2" s="267"/>
-      <c r="G2" s="267"/>
-      <c r="H2" s="267"/>
-      <c r="I2" s="267"/>
-      <c r="J2" s="267"/>
-      <c r="K2" s="267"/>
-      <c r="L2" s="267"/>
-      <c r="M2" s="267"/>
-      <c r="N2" s="267"/>
-      <c r="O2" s="267"/>
-      <c r="P2" s="267"/>
-      <c r="Q2" s="267"/>
-      <c r="R2" s="267"/>
-      <c r="S2" s="267"/>
-      <c r="T2" s="267"/>
-      <c r="U2" s="267"/>
-      <c r="V2" s="267"/>
-      <c r="W2" s="267"/>
-      <c r="X2" s="267"/>
-      <c r="Y2" s="267"/>
-      <c r="Z2" s="267"/>
+      <c r="B2" s="263"/>
+      <c r="C2" s="263"/>
+      <c r="D2" s="263"/>
+      <c r="E2" s="263"/>
+      <c r="F2" s="263"/>
+      <c r="G2" s="263"/>
+      <c r="H2" s="263"/>
+      <c r="I2" s="263"/>
+      <c r="J2" s="263"/>
+      <c r="K2" s="263"/>
+      <c r="L2" s="263"/>
+      <c r="M2" s="263"/>
+      <c r="N2" s="263"/>
+      <c r="O2" s="263"/>
+      <c r="P2" s="263"/>
+      <c r="Q2" s="263"/>
+      <c r="R2" s="263"/>
+      <c r="S2" s="263"/>
+      <c r="T2" s="263"/>
+      <c r="U2" s="263"/>
+      <c r="V2" s="263"/>
+      <c r="W2" s="263"/>
+      <c r="X2" s="263"/>
+      <c r="Y2" s="263"/>
+      <c r="Z2" s="263"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.15">
       <c r="C3" s="119" t="s">
@@ -17255,10 +17320,10 @@
       <c r="E5" s="260"/>
       <c r="F5" s="260"/>
       <c r="G5" s="260"/>
-      <c r="AC5" s="268" t="s">
+      <c r="AC5" s="264" t="s">
         <v>161</v>
       </c>
-      <c r="AD5" s="269"/>
+      <c r="AD5" s="265"/>
       <c r="AE5" s="119"/>
       <c r="AF5" s="119"/>
     </row>
@@ -17635,10 +17700,10 @@
       </c>
       <c r="D21" s="262"/>
       <c r="E21" s="262"/>
-      <c r="T21" s="263" t="s">
+      <c r="T21" s="266" t="s">
         <v>163</v>
       </c>
-      <c r="U21" s="264"/>
+      <c r="U21" s="267"/>
       <c r="V21" s="167" t="s">
         <v>154</v>
       </c>
@@ -17647,17 +17712,17 @@
       </c>
       <c r="X21" s="128"/>
       <c r="Y21" s="128"/>
-      <c r="Z21" s="265" t="s">
+      <c r="Z21" s="268" t="s">
         <v>157</v>
       </c>
-      <c r="AA21" s="265"/>
-      <c r="AB21" s="265"/>
+      <c r="AA21" s="268"/>
+      <c r="AB21" s="268"/>
     </row>
     <row r="22" spans="1:34" ht="15" x14ac:dyDescent="0.15">
-      <c r="A22" s="263" t="s">
+      <c r="A22" s="266" t="s">
         <v>153</v>
       </c>
-      <c r="B22" s="264"/>
+      <c r="B22" s="267"/>
       <c r="C22" s="133" t="s">
         <v>8</v>
       </c>
@@ -17709,10 +17774,10 @@
       <c r="S22" s="168" t="s">
         <v>176</v>
       </c>
-      <c r="T22" s="263" t="s">
+      <c r="T22" s="266" t="s">
         <v>188</v>
       </c>
-      <c r="U22" s="266"/>
+      <c r="U22" s="269"/>
       <c r="V22" s="168" t="s">
         <v>182</v>
       </c>
@@ -18421,17 +18486,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="T21:U21"/>
+    <mergeCell ref="Z21:AB21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="T22:U22"/>
     <mergeCell ref="T20:AB20"/>
     <mergeCell ref="A1:Z1"/>
     <mergeCell ref="A2:Z2"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="AC5:AD5"/>
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="T21:U21"/>
-    <mergeCell ref="Z21:AB21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="T22:U22"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X13 T32 T25:T28" xr:uid="{A3DEBC13-46CE-4D1E-BD8D-45F2ED5DBE94}">
@@ -18481,54 +18546,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.15">
-      <c r="A1" s="267" t="s">
+      <c r="A1" s="263" t="s">
         <v>151</v>
       </c>
-      <c r="B1" s="267"/>
-      <c r="C1" s="267"/>
-      <c r="D1" s="267"/>
-      <c r="E1" s="267"/>
-      <c r="F1" s="267"/>
-      <c r="G1" s="267"/>
-      <c r="H1" s="267"/>
-      <c r="I1" s="267"/>
-      <c r="J1" s="267"/>
-      <c r="K1" s="267"/>
-      <c r="L1" s="267"/>
-      <c r="M1" s="267"/>
-      <c r="N1" s="267"/>
-      <c r="O1" s="267"/>
-      <c r="P1" s="267"/>
-      <c r="Q1" s="267"/>
-      <c r="R1" s="267"/>
-      <c r="S1" s="267"/>
-      <c r="T1" s="267"/>
-      <c r="U1" s="267"/>
+      <c r="B1" s="263"/>
+      <c r="C1" s="263"/>
+      <c r="D1" s="263"/>
+      <c r="E1" s="263"/>
+      <c r="F1" s="263"/>
+      <c r="G1" s="263"/>
+      <c r="H1" s="263"/>
+      <c r="I1" s="263"/>
+      <c r="J1" s="263"/>
+      <c r="K1" s="263"/>
+      <c r="L1" s="263"/>
+      <c r="M1" s="263"/>
+      <c r="N1" s="263"/>
+      <c r="O1" s="263"/>
+      <c r="P1" s="263"/>
+      <c r="Q1" s="263"/>
+      <c r="R1" s="263"/>
+      <c r="S1" s="263"/>
+      <c r="T1" s="263"/>
+      <c r="U1" s="263"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.15">
-      <c r="A2" s="267" t="s">
+      <c r="A2" s="263" t="s">
         <v>150</v>
       </c>
-      <c r="B2" s="267"/>
-      <c r="C2" s="267"/>
-      <c r="D2" s="267"/>
-      <c r="E2" s="267"/>
-      <c r="F2" s="267"/>
-      <c r="G2" s="267"/>
-      <c r="H2" s="267"/>
-      <c r="I2" s="267"/>
-      <c r="J2" s="267"/>
-      <c r="K2" s="267"/>
-      <c r="L2" s="267"/>
-      <c r="M2" s="267"/>
-      <c r="N2" s="267"/>
-      <c r="O2" s="267"/>
-      <c r="P2" s="267"/>
-      <c r="Q2" s="267"/>
-      <c r="R2" s="267"/>
-      <c r="S2" s="267"/>
-      <c r="T2" s="267"/>
-      <c r="U2" s="267"/>
+      <c r="B2" s="263"/>
+      <c r="C2" s="263"/>
+      <c r="D2" s="263"/>
+      <c r="E2" s="263"/>
+      <c r="F2" s="263"/>
+      <c r="G2" s="263"/>
+      <c r="H2" s="263"/>
+      <c r="I2" s="263"/>
+      <c r="J2" s="263"/>
+      <c r="K2" s="263"/>
+      <c r="L2" s="263"/>
+      <c r="M2" s="263"/>
+      <c r="N2" s="263"/>
+      <c r="O2" s="263"/>
+      <c r="P2" s="263"/>
+      <c r="Q2" s="263"/>
+      <c r="R2" s="263"/>
+      <c r="S2" s="263"/>
+      <c r="T2" s="263"/>
+      <c r="U2" s="263"/>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.15">
       <c r="C3" s="119" t="s">
@@ -18545,10 +18610,10 @@
       <c r="E5" s="260"/>
       <c r="F5" s="260"/>
       <c r="G5" s="260"/>
-      <c r="X5" s="268" t="s">
+      <c r="X5" s="264" t="s">
         <v>161</v>
       </c>
-      <c r="Y5" s="269"/>
+      <c r="Y5" s="265"/>
       <c r="Z5" s="119"/>
       <c r="AA5" s="119"/>
     </row>
@@ -18882,10 +18947,10 @@
       </c>
       <c r="D21" s="262"/>
       <c r="E21" s="262"/>
-      <c r="O21" s="263" t="s">
+      <c r="O21" s="266" t="s">
         <v>163</v>
       </c>
-      <c r="P21" s="264"/>
+      <c r="P21" s="267"/>
       <c r="Q21" s="167" t="s">
         <v>154</v>
       </c>
@@ -18894,17 +18959,17 @@
       </c>
       <c r="S21" s="128"/>
       <c r="T21" s="128"/>
-      <c r="U21" s="265" t="s">
+      <c r="U21" s="268" t="s">
         <v>157</v>
       </c>
-      <c r="V21" s="265"/>
-      <c r="W21" s="265"/>
+      <c r="V21" s="268"/>
+      <c r="W21" s="268"/>
     </row>
     <row r="22" spans="1:23" ht="15" x14ac:dyDescent="0.15">
-      <c r="A22" s="263" t="s">
+      <c r="A22" s="266" t="s">
         <v>153</v>
       </c>
-      <c r="B22" s="264"/>
+      <c r="B22" s="267"/>
       <c r="C22" s="133" t="s">
         <v>8</v>
       </c>
@@ -18941,10 +19006,10 @@
       <c r="N22" s="168" t="s">
         <v>176</v>
       </c>
-      <c r="O22" s="263" t="s">
+      <c r="O22" s="266" t="s">
         <v>188</v>
       </c>
-      <c r="P22" s="266"/>
+      <c r="P22" s="269"/>
       <c r="Q22" s="168" t="s">
         <v>182</v>
       </c>
@@ -21490,17 +21555,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="U21:W21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="O22:P22"/>
     <mergeCell ref="O20:W20"/>
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="X5:Y5"/>
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="U21:W21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="O22:P22"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S13 O25:O34 O36:O37 O40:O47 O50:O57" xr:uid="{664F27CC-03B8-41DD-9E77-6535CBE6D30A}">

</xml_diff>

<commit_message>
Measurement Type update results in Results update.
Save Measurement Type settings in the saved measurements and restore them.
Fixed problem with Results Window not appearing on MacOS.

Make sure that the apply from the settings window updates the results.
Save new testcases with the missing information added.
</commit_message>
<xml_diff>
--- a/Wood Property Measurementsl.xlsx
+++ b/Wood Property Measurementsl.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dws/src/GuitarTap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDAFE4A1-AE11-E147-8908-5D845CA52936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1B7EEE-79AF-A44D-8409-860EB9189235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="660" windowWidth="30240" windowHeight="16640" tabRatio="768" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="16640" tabRatio="768" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monopole Mobility" sheetId="10" r:id="rId1"/>
@@ -104,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="266">
   <si>
     <t>E</t>
   </si>
@@ -2916,16 +2916,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2940,14 +2949,8 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2972,9 +2975,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -13720,22 +13720,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{FE1B2129-DF31-44E8-8E35-33B39C225DCE}" name="Vib_Stiff24" displayName="Vib_Stiff24" ref="AC6:AD10" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{FE1B2129-DF31-44E8-8E35-33B39C225DCE}" name="Vib_Stiff24" displayName="Vib_Stiff24" ref="AC6:AD10" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
   <autoFilter ref="AC6:AD10" xr:uid="{42B488F6-5D03-4246-8503-BE308C80AAA5}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{A7988C3C-FFDF-4367-8118-CFE4FAB58656}" name="PanelType" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{AC9FD991-01A9-4D4B-8EA2-F97B127BFFA2}" name="Value" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{A7988C3C-FFDF-4367-8118-CFE4FAB58656}" name="PanelType" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{AC9FD991-01A9-4D4B-8EA2-F97B127BFFA2}" name="Value" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8FFEEA05-A23C-446D-8F23-10CBD8852EB9}" name="Vib_Stiff2" displayName="Vib_Stiff2" ref="X6:Y10" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8FFEEA05-A23C-446D-8F23-10CBD8852EB9}" name="Vib_Stiff2" displayName="Vib_Stiff2" ref="X6:Y10" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
   <autoFilter ref="X6:Y10" xr:uid="{42B488F6-5D03-4246-8503-BE308C80AAA5}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{8C12DDF7-C9B2-458A-A55F-9601B9FB8147}" name="PanelType" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{7B5557FB-886A-49CD-8245-B4A260F460A3}" name="Value" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{8C12DDF7-C9B2-458A-A55F-9601B9FB8147}" name="PanelType" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{7B5557FB-886A-49CD-8245-B4A260F460A3}" name="Value" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -14669,7 +14669,7 @@
     </row>
     <row r="16" spans="2:2" ht="14" thickBot="1" x14ac:dyDescent="0.2"/>
     <row r="17" spans="2:25" ht="42" x14ac:dyDescent="0.15">
-      <c r="B17" s="277" t="s">
+      <c r="B17" s="278" t="s">
         <v>214</v>
       </c>
       <c r="C17" s="197" t="s">
@@ -14704,7 +14704,7 @@
       </c>
     </row>
     <row r="18" spans="2:25" ht="14" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="278"/>
+      <c r="B18" s="279"/>
       <c r="C18" s="202" t="s">
         <v>217</v>
       </c>
@@ -14946,10 +14946,10 @@
     </row>
     <row r="26" spans="2:25" ht="14" thickBot="1" x14ac:dyDescent="0.2"/>
     <row r="27" spans="2:25" ht="14" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="275" t="s">
+      <c r="B27" s="276" t="s">
         <v>255</v>
       </c>
-      <c r="C27" s="276"/>
+      <c r="C27" s="277"/>
     </row>
     <row r="28" spans="2:25" ht="28" x14ac:dyDescent="0.15">
       <c r="B28" s="257" t="s">
@@ -14976,18 +14976,18 @@
     </row>
     <row r="30" spans="2:25" ht="14" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B30" s="109"/>
-      <c r="C30" s="271" t="s">
+      <c r="C30" s="272" t="s">
         <v>236</v>
       </c>
-      <c r="D30" s="272"/>
-      <c r="E30" s="272"/>
-      <c r="F30" s="272"/>
-      <c r="G30" s="272"/>
-      <c r="H30" s="272"/>
-      <c r="I30" s="272"/>
-      <c r="J30" s="272"/>
-      <c r="K30" s="272"/>
-      <c r="L30" s="273"/>
+      <c r="D30" s="273"/>
+      <c r="E30" s="273"/>
+      <c r="F30" s="273"/>
+      <c r="G30" s="273"/>
+      <c r="H30" s="273"/>
+      <c r="I30" s="273"/>
+      <c r="J30" s="273"/>
+      <c r="K30" s="273"/>
+      <c r="L30" s="274"/>
       <c r="M30" s="224" t="s">
         <v>238</v>
       </c>
@@ -14996,11 +14996,11 @@
       <c r="R30" s="109"/>
       <c r="S30" s="109"/>
       <c r="T30" s="109"/>
-      <c r="U30" s="274"/>
-      <c r="V30" s="274"/>
-      <c r="W30" s="274"/>
-      <c r="X30" s="274"/>
-      <c r="Y30" s="274"/>
+      <c r="U30" s="275"/>
+      <c r="V30" s="275"/>
+      <c r="W30" s="275"/>
+      <c r="X30" s="275"/>
+      <c r="Y30" s="275"/>
     </row>
     <row r="31" spans="2:25" ht="42" x14ac:dyDescent="0.15">
       <c r="B31" s="109"/>
@@ -16774,11 +16774,11 @@
       <c r="C5" s="12"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.15">
-      <c r="G10" s="262" t="s">
+      <c r="G10" s="271" t="s">
         <v>148</v>
       </c>
-      <c r="H10" s="262"/>
-      <c r="I10" s="262"/>
+      <c r="H10" s="271"/>
+      <c r="I10" s="271"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.15">
       <c r="C11" s="41" t="s">
@@ -16957,19 +16957,19 @@
     </row>
     <row r="21" spans="3:10" ht="14" thickBot="1" x14ac:dyDescent="0.2"/>
     <row r="22" spans="3:10" ht="14" thickTop="1" x14ac:dyDescent="0.15">
-      <c r="C22" s="261" t="s">
+      <c r="C22" s="263" t="s">
         <v>119</v>
       </c>
-      <c r="D22" s="261"/>
-      <c r="E22" s="261"/>
-      <c r="F22" s="261"/>
-      <c r="G22" s="261"/>
+      <c r="D22" s="263"/>
+      <c r="E22" s="263"/>
+      <c r="F22" s="263"/>
+      <c r="G22" s="263"/>
     </row>
     <row r="23" spans="3:10" x14ac:dyDescent="0.15">
-      <c r="C23" s="260" t="s">
+      <c r="C23" s="266" t="s">
         <v>127</v>
       </c>
-      <c r="D23" s="260"/>
+      <c r="D23" s="266"/>
       <c r="E23" s="111" t="s">
         <v>133</v>
       </c>
@@ -17252,64 +17252,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.15">
-      <c r="A1" s="268" t="s">
+      <c r="A1" s="262" t="s">
         <v>195</v>
       </c>
-      <c r="B1" s="268"/>
-      <c r="C1" s="268"/>
-      <c r="D1" s="268"/>
-      <c r="E1" s="268"/>
-      <c r="F1" s="268"/>
-      <c r="G1" s="268"/>
-      <c r="H1" s="268"/>
-      <c r="I1" s="268"/>
-      <c r="J1" s="268"/>
-      <c r="K1" s="268"/>
-      <c r="L1" s="268"/>
-      <c r="M1" s="268"/>
-      <c r="N1" s="268"/>
-      <c r="O1" s="268"/>
-      <c r="P1" s="268"/>
-      <c r="Q1" s="268"/>
-      <c r="R1" s="268"/>
-      <c r="S1" s="268"/>
-      <c r="T1" s="268"/>
-      <c r="U1" s="268"/>
-      <c r="V1" s="268"/>
-      <c r="W1" s="268"/>
-      <c r="X1" s="268"/>
-      <c r="Y1" s="268"/>
-      <c r="Z1" s="268"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
+      <c r="H1" s="262"/>
+      <c r="I1" s="262"/>
+      <c r="J1" s="262"/>
+      <c r="K1" s="262"/>
+      <c r="L1" s="262"/>
+      <c r="M1" s="262"/>
+      <c r="N1" s="262"/>
+      <c r="O1" s="262"/>
+      <c r="P1" s="262"/>
+      <c r="Q1" s="262"/>
+      <c r="R1" s="262"/>
+      <c r="S1" s="262"/>
+      <c r="T1" s="262"/>
+      <c r="U1" s="262"/>
+      <c r="V1" s="262"/>
+      <c r="W1" s="262"/>
+      <c r="X1" s="262"/>
+      <c r="Y1" s="262"/>
+      <c r="Z1" s="262"/>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.15">
-      <c r="A2" s="268" t="s">
+      <c r="A2" s="262" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="268"/>
-      <c r="C2" s="268"/>
-      <c r="D2" s="268"/>
-      <c r="E2" s="268"/>
-      <c r="F2" s="268"/>
-      <c r="G2" s="268"/>
-      <c r="H2" s="268"/>
-      <c r="I2" s="268"/>
-      <c r="J2" s="268"/>
-      <c r="K2" s="268"/>
-      <c r="L2" s="268"/>
-      <c r="M2" s="268"/>
-      <c r="N2" s="268"/>
-      <c r="O2" s="268"/>
-      <c r="P2" s="268"/>
-      <c r="Q2" s="268"/>
-      <c r="R2" s="268"/>
-      <c r="S2" s="268"/>
-      <c r="T2" s="268"/>
-      <c r="U2" s="268"/>
-      <c r="V2" s="268"/>
-      <c r="W2" s="268"/>
-      <c r="X2" s="268"/>
-      <c r="Y2" s="268"/>
-      <c r="Z2" s="268"/>
+      <c r="B2" s="262"/>
+      <c r="C2" s="262"/>
+      <c r="D2" s="262"/>
+      <c r="E2" s="262"/>
+      <c r="F2" s="262"/>
+      <c r="G2" s="262"/>
+      <c r="H2" s="262"/>
+      <c r="I2" s="262"/>
+      <c r="J2" s="262"/>
+      <c r="K2" s="262"/>
+      <c r="L2" s="262"/>
+      <c r="M2" s="262"/>
+      <c r="N2" s="262"/>
+      <c r="O2" s="262"/>
+      <c r="P2" s="262"/>
+      <c r="Q2" s="262"/>
+      <c r="R2" s="262"/>
+      <c r="S2" s="262"/>
+      <c r="T2" s="262"/>
+      <c r="U2" s="262"/>
+      <c r="V2" s="262"/>
+      <c r="W2" s="262"/>
+      <c r="X2" s="262"/>
+      <c r="Y2" s="262"/>
+      <c r="Z2" s="262"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.15">
       <c r="C3" s="119" t="s">
@@ -17319,25 +17319,25 @@
     </row>
     <row r="4" spans="1:32" ht="14" thickBot="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:32" ht="14" thickTop="1" x14ac:dyDescent="0.15">
-      <c r="C5" s="261" t="s">
+      <c r="C5" s="263" t="s">
         <v>119</v>
       </c>
-      <c r="D5" s="261"/>
-      <c r="E5" s="261"/>
-      <c r="F5" s="261"/>
-      <c r="G5" s="261"/>
-      <c r="AC5" s="269" t="s">
+      <c r="D5" s="263"/>
+      <c r="E5" s="263"/>
+      <c r="F5" s="263"/>
+      <c r="G5" s="263"/>
+      <c r="AC5" s="264" t="s">
         <v>161</v>
       </c>
-      <c r="AD5" s="270"/>
+      <c r="AD5" s="265"/>
       <c r="AE5" s="119"/>
       <c r="AF5" s="119"/>
     </row>
     <row r="6" spans="1:32" ht="15" x14ac:dyDescent="0.15">
-      <c r="C6" s="260" t="s">
+      <c r="C6" s="266" t="s">
         <v>127</v>
       </c>
-      <c r="D6" s="260"/>
+      <c r="D6" s="266"/>
       <c r="E6" s="166" t="s">
         <v>177</v>
       </c>
@@ -17688,28 +17688,28 @@
       <c r="O19" s="175"/>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.15">
-      <c r="T20" s="263" t="s">
+      <c r="T20" s="261" t="s">
         <v>160</v>
       </c>
-      <c r="U20" s="263"/>
-      <c r="V20" s="263"/>
-      <c r="W20" s="263"/>
-      <c r="X20" s="263"/>
-      <c r="Y20" s="263"/>
-      <c r="Z20" s="263"/>
-      <c r="AA20" s="263"/>
-      <c r="AB20" s="263"/>
+      <c r="U20" s="261"/>
+      <c r="V20" s="261"/>
+      <c r="W20" s="261"/>
+      <c r="X20" s="261"/>
+      <c r="Y20" s="261"/>
+      <c r="Z20" s="261"/>
+      <c r="AA20" s="261"/>
+      <c r="AB20" s="261"/>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.15">
-      <c r="C21" s="263" t="s">
+      <c r="C21" s="261" t="s">
         <v>148</v>
       </c>
-      <c r="D21" s="263"/>
-      <c r="E21" s="263"/>
-      <c r="T21" s="264" t="s">
+      <c r="D21" s="261"/>
+      <c r="E21" s="261"/>
+      <c r="T21" s="267" t="s">
         <v>163</v>
       </c>
-      <c r="U21" s="265"/>
+      <c r="U21" s="268"/>
       <c r="V21" s="167" t="s">
         <v>154</v>
       </c>
@@ -17718,17 +17718,17 @@
       </c>
       <c r="X21" s="128"/>
       <c r="Y21" s="128"/>
-      <c r="Z21" s="266" t="s">
+      <c r="Z21" s="269" t="s">
         <v>157</v>
       </c>
-      <c r="AA21" s="266"/>
-      <c r="AB21" s="266"/>
+      <c r="AA21" s="269"/>
+      <c r="AB21" s="269"/>
     </row>
     <row r="22" spans="1:34" ht="15" x14ac:dyDescent="0.15">
-      <c r="A22" s="264" t="s">
+      <c r="A22" s="267" t="s">
         <v>153</v>
       </c>
-      <c r="B22" s="265"/>
+      <c r="B22" s="268"/>
       <c r="C22" s="133" t="s">
         <v>8</v>
       </c>
@@ -17780,10 +17780,10 @@
       <c r="S22" s="168" t="s">
         <v>176</v>
       </c>
-      <c r="T22" s="264" t="s">
+      <c r="T22" s="267" t="s">
         <v>188</v>
       </c>
-      <c r="U22" s="267"/>
+      <c r="U22" s="270"/>
       <c r="V22" s="168" t="s">
         <v>182</v>
       </c>
@@ -18492,17 +18492,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="T21:U21"/>
+    <mergeCell ref="Z21:AB21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="T22:U22"/>
     <mergeCell ref="T20:AB20"/>
     <mergeCell ref="A1:Z1"/>
     <mergeCell ref="A2:Z2"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="AC5:AD5"/>
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="T21:U21"/>
-    <mergeCell ref="Z21:AB21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="T22:U22"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X13 T32 T25:T28" xr:uid="{A3DEBC13-46CE-4D1E-BD8D-45F2ED5DBE94}">
@@ -18552,54 +18552,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.15">
-      <c r="A1" s="268" t="s">
+      <c r="A1" s="262" t="s">
         <v>151</v>
       </c>
-      <c r="B1" s="268"/>
-      <c r="C1" s="268"/>
-      <c r="D1" s="268"/>
-      <c r="E1" s="268"/>
-      <c r="F1" s="268"/>
-      <c r="G1" s="268"/>
-      <c r="H1" s="268"/>
-      <c r="I1" s="268"/>
-      <c r="J1" s="268"/>
-      <c r="K1" s="268"/>
-      <c r="L1" s="268"/>
-      <c r="M1" s="268"/>
-      <c r="N1" s="268"/>
-      <c r="O1" s="268"/>
-      <c r="P1" s="268"/>
-      <c r="Q1" s="268"/>
-      <c r="R1" s="268"/>
-      <c r="S1" s="268"/>
-      <c r="T1" s="268"/>
-      <c r="U1" s="268"/>
+      <c r="B1" s="262"/>
+      <c r="C1" s="262"/>
+      <c r="D1" s="262"/>
+      <c r="E1" s="262"/>
+      <c r="F1" s="262"/>
+      <c r="G1" s="262"/>
+      <c r="H1" s="262"/>
+      <c r="I1" s="262"/>
+      <c r="J1" s="262"/>
+      <c r="K1" s="262"/>
+      <c r="L1" s="262"/>
+      <c r="M1" s="262"/>
+      <c r="N1" s="262"/>
+      <c r="O1" s="262"/>
+      <c r="P1" s="262"/>
+      <c r="Q1" s="262"/>
+      <c r="R1" s="262"/>
+      <c r="S1" s="262"/>
+      <c r="T1" s="262"/>
+      <c r="U1" s="262"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.15">
-      <c r="A2" s="268" t="s">
+      <c r="A2" s="262" t="s">
         <v>150</v>
       </c>
-      <c r="B2" s="268"/>
-      <c r="C2" s="268"/>
-      <c r="D2" s="268"/>
-      <c r="E2" s="268"/>
-      <c r="F2" s="268"/>
-      <c r="G2" s="268"/>
-      <c r="H2" s="268"/>
-      <c r="I2" s="268"/>
-      <c r="J2" s="268"/>
-      <c r="K2" s="268"/>
-      <c r="L2" s="268"/>
-      <c r="M2" s="268"/>
-      <c r="N2" s="268"/>
-      <c r="O2" s="268"/>
-      <c r="P2" s="268"/>
-      <c r="Q2" s="268"/>
-      <c r="R2" s="268"/>
-      <c r="S2" s="268"/>
-      <c r="T2" s="268"/>
-      <c r="U2" s="268"/>
+      <c r="B2" s="262"/>
+      <c r="C2" s="262"/>
+      <c r="D2" s="262"/>
+      <c r="E2" s="262"/>
+      <c r="F2" s="262"/>
+      <c r="G2" s="262"/>
+      <c r="H2" s="262"/>
+      <c r="I2" s="262"/>
+      <c r="J2" s="262"/>
+      <c r="K2" s="262"/>
+      <c r="L2" s="262"/>
+      <c r="M2" s="262"/>
+      <c r="N2" s="262"/>
+      <c r="O2" s="262"/>
+      <c r="P2" s="262"/>
+      <c r="Q2" s="262"/>
+      <c r="R2" s="262"/>
+      <c r="S2" s="262"/>
+      <c r="T2" s="262"/>
+      <c r="U2" s="262"/>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.15">
       <c r="C3" s="119" t="s">
@@ -18609,25 +18609,25 @@
     </row>
     <row r="4" spans="1:27" ht="14" thickBot="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:27" ht="14" thickTop="1" x14ac:dyDescent="0.15">
-      <c r="C5" s="261" t="s">
+      <c r="C5" s="263" t="s">
         <v>119</v>
       </c>
-      <c r="D5" s="261"/>
-      <c r="E5" s="261"/>
-      <c r="F5" s="261"/>
-      <c r="G5" s="261"/>
-      <c r="X5" s="269" t="s">
+      <c r="D5" s="263"/>
+      <c r="E5" s="263"/>
+      <c r="F5" s="263"/>
+      <c r="G5" s="263"/>
+      <c r="X5" s="264" t="s">
         <v>161</v>
       </c>
-      <c r="Y5" s="270"/>
+      <c r="Y5" s="265"/>
       <c r="Z5" s="119"/>
       <c r="AA5" s="119"/>
     </row>
     <row r="6" spans="1:27" ht="15" x14ac:dyDescent="0.15">
-      <c r="C6" s="260" t="s">
+      <c r="C6" s="266" t="s">
         <v>127</v>
       </c>
-      <c r="D6" s="260"/>
+      <c r="D6" s="266"/>
       <c r="E6" s="166" t="s">
         <v>177</v>
       </c>
@@ -18935,28 +18935,28 @@
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.15">
-      <c r="O20" s="263" t="s">
+      <c r="O20" s="261" t="s">
         <v>160</v>
       </c>
-      <c r="P20" s="263"/>
-      <c r="Q20" s="263"/>
-      <c r="R20" s="263"/>
-      <c r="S20" s="263"/>
-      <c r="T20" s="263"/>
-      <c r="U20" s="263"/>
-      <c r="V20" s="263"/>
-      <c r="W20" s="263"/>
+      <c r="P20" s="261"/>
+      <c r="Q20" s="261"/>
+      <c r="R20" s="261"/>
+      <c r="S20" s="261"/>
+      <c r="T20" s="261"/>
+      <c r="U20" s="261"/>
+      <c r="V20" s="261"/>
+      <c r="W20" s="261"/>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.15">
-      <c r="C21" s="263" t="s">
+      <c r="C21" s="261" t="s">
         <v>148</v>
       </c>
-      <c r="D21" s="263"/>
-      <c r="E21" s="263"/>
-      <c r="O21" s="264" t="s">
+      <c r="D21" s="261"/>
+      <c r="E21" s="261"/>
+      <c r="O21" s="267" t="s">
         <v>163</v>
       </c>
-      <c r="P21" s="265"/>
+      <c r="P21" s="268"/>
       <c r="Q21" s="167" t="s">
         <v>154</v>
       </c>
@@ -18965,17 +18965,17 @@
       </c>
       <c r="S21" s="128"/>
       <c r="T21" s="128"/>
-      <c r="U21" s="266" t="s">
+      <c r="U21" s="269" t="s">
         <v>157</v>
       </c>
-      <c r="V21" s="266"/>
-      <c r="W21" s="266"/>
+      <c r="V21" s="269"/>
+      <c r="W21" s="269"/>
     </row>
     <row r="22" spans="1:23" ht="15" x14ac:dyDescent="0.15">
-      <c r="A22" s="264" t="s">
+      <c r="A22" s="267" t="s">
         <v>153</v>
       </c>
-      <c r="B22" s="265"/>
+      <c r="B22" s="268"/>
       <c r="C22" s="133" t="s">
         <v>8</v>
       </c>
@@ -19012,10 +19012,10 @@
       <c r="N22" s="168" t="s">
         <v>176</v>
       </c>
-      <c r="O22" s="264" t="s">
+      <c r="O22" s="267" t="s">
         <v>188</v>
       </c>
-      <c r="P22" s="267"/>
+      <c r="P22" s="270"/>
       <c r="Q22" s="168" t="s">
         <v>182</v>
       </c>
@@ -20868,7 +20868,7 @@
         <v>0.39800000000000002</v>
       </c>
       <c r="G50" s="153">
-        <f t="shared" ref="G50:G57" si="20">F50/(C50*D50*E50)</f>
+        <f t="shared" ref="G50:G56" si="20">F50/(C50*D50*E50)</f>
         <v>824.16399123984093</v>
       </c>
       <c r="H50" s="156">
@@ -21527,7 +21527,7 @@
       </c>
     </row>
     <row r="60" spans="1:23" x14ac:dyDescent="0.15">
-      <c r="B60" s="279" t="s">
+      <c r="B60" s="260" t="s">
         <v>265</v>
       </c>
       <c r="C60" s="109">
@@ -21546,43 +21546,55 @@
         <f>F60/(C60*D60*E60)</f>
         <v>348.87361937825227</v>
       </c>
+      <c r="H60" s="109">
+        <v>67.400000000000006</v>
+      </c>
+      <c r="I60" s="109">
+        <v>117.5</v>
+      </c>
+      <c r="J60" s="109">
+        <v>54.8</v>
+      </c>
       <c r="K60" s="139">
         <f t="shared" ref="K60" si="30">Coef_1*G60*C60^4*H60^2/E60^2/10^9</f>
-        <v>0</v>
+        <v>6.1275443748904177</v>
       </c>
       <c r="L60" s="138">
         <f t="shared" ref="L60" si="31">Coef_1*G60*D60^4*I60^2/E60^2/10^9</f>
-        <v>0</v>
-      </c>
-      <c r="M60" s="140" t="e">
+        <v>0.45571916558324194</v>
+      </c>
+      <c r="M60" s="140">
         <f t="shared" ref="M60" si="32">K60/L60</f>
-        <v>#DIV/0!</v>
+        <v>13.445878158422891</v>
       </c>
       <c r="N60" s="138">
         <f t="shared" ref="N60" si="33">(3*(1/(PI()/2)^2)*G60*C60^2*D60^2*J60^2/E60^2)/10^9</f>
-        <v>0</v>
-      </c>
-      <c r="P60" s="140" t="e">
+        <v>0.81834079619638811</v>
+      </c>
+      <c r="O60" s="121" t="s">
+        <v>146</v>
+      </c>
+      <c r="P60" s="140">
         <f>INDEX(Vib_Stiff2[],MATCH($O60,Vib_Stiff2[PanelType],0),2)</f>
-        <v>#N/A</v>
+        <v>60</v>
       </c>
       <c r="Q60" s="109">
         <v>0.49</v>
       </c>
       <c r="R60" s="109">
-        <v>0.36799999999999999</v>
-      </c>
-      <c r="S60" s="140" t="e">
+        <v>0.39</v>
+      </c>
+      <c r="S60" s="140">
         <f t="shared" ref="S60" si="34">Coef_2*P60*Q60^2*G60^0.5</f>
-        <v>#N/A</v>
+        <v>258.25321505789361</v>
       </c>
       <c r="T60" s="142">
         <f t="shared" ref="T60" si="35">(K60+(Q60/R60)^4*L60+(Q60/R60)^2*(Coef_3*K60+Coef_4*N60))*10^9</f>
-        <v>0</v>
-      </c>
-      <c r="U60" s="158" t="e">
+        <v>8986324784.4693947</v>
+      </c>
+      <c r="U60" s="158">
         <f t="shared" ref="U60" si="36">S60/T60^0.5*1000</f>
-        <v>#N/A</v>
+        <v>2.72429843832326</v>
       </c>
     </row>
     <row r="66" spans="9:15" x14ac:dyDescent="0.15">
@@ -21620,20 +21632,20 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="U21:W21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="O22:P22"/>
     <mergeCell ref="O20:W20"/>
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="X5:Y5"/>
     <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="U21:W21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="O22:P22"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S13 O25:O34 O36:O37 O40:O47 O50:O57" xr:uid="{664F27CC-03B8-41DD-9E77-6535CBE6D30A}">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S13 O25:O34 O36:O37 O40:O47 O50:O57 O60" xr:uid="{664F27CC-03B8-41DD-9E77-6535CBE6D30A}">
       <formula1>dd_items</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fixed brace and plate measurements (again).
</commit_message>
<xml_diff>
--- a/Wood Property Measurementsl.xlsx
+++ b/Wood Property Measurementsl.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dws/src/GuitarTap/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1B7EEE-79AF-A44D-8409-860EB9189235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B802DA3F-165E-3F45-81E6-A4A549B913C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="16640" tabRatio="768" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="960" windowWidth="30240" windowHeight="16640" tabRatio="768" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monopole Mobility" sheetId="10" r:id="rId1"/>
@@ -2922,6 +2922,18 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -2935,18 +2947,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -16957,19 +16957,19 @@
     </row>
     <row r="21" spans="3:10" ht="14" thickBot="1" x14ac:dyDescent="0.2"/>
     <row r="22" spans="3:10" ht="14" thickTop="1" x14ac:dyDescent="0.15">
-      <c r="C22" s="263" t="s">
+      <c r="C22" s="267" t="s">
         <v>119</v>
       </c>
-      <c r="D22" s="263"/>
-      <c r="E22" s="263"/>
-      <c r="F22" s="263"/>
-      <c r="G22" s="263"/>
+      <c r="D22" s="267"/>
+      <c r="E22" s="267"/>
+      <c r="F22" s="267"/>
+      <c r="G22" s="267"/>
     </row>
     <row r="23" spans="3:10" x14ac:dyDescent="0.15">
-      <c r="C23" s="266" t="s">
+      <c r="C23" s="270" t="s">
         <v>127</v>
       </c>
-      <c r="D23" s="266"/>
+      <c r="D23" s="270"/>
       <c r="E23" s="111" t="s">
         <v>133</v>
       </c>
@@ -17252,64 +17252,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:32" x14ac:dyDescent="0.15">
-      <c r="A1" s="262" t="s">
+      <c r="A1" s="266" t="s">
         <v>195</v>
       </c>
-      <c r="B1" s="262"/>
-      <c r="C1" s="262"/>
-      <c r="D1" s="262"/>
-      <c r="E1" s="262"/>
-      <c r="F1" s="262"/>
-      <c r="G1" s="262"/>
-      <c r="H1" s="262"/>
-      <c r="I1" s="262"/>
-      <c r="J1" s="262"/>
-      <c r="K1" s="262"/>
-      <c r="L1" s="262"/>
-      <c r="M1" s="262"/>
-      <c r="N1" s="262"/>
-      <c r="O1" s="262"/>
-      <c r="P1" s="262"/>
-      <c r="Q1" s="262"/>
-      <c r="R1" s="262"/>
-      <c r="S1" s="262"/>
-      <c r="T1" s="262"/>
-      <c r="U1" s="262"/>
-      <c r="V1" s="262"/>
-      <c r="W1" s="262"/>
-      <c r="X1" s="262"/>
-      <c r="Y1" s="262"/>
-      <c r="Z1" s="262"/>
+      <c r="B1" s="266"/>
+      <c r="C1" s="266"/>
+      <c r="D1" s="266"/>
+      <c r="E1" s="266"/>
+      <c r="F1" s="266"/>
+      <c r="G1" s="266"/>
+      <c r="H1" s="266"/>
+      <c r="I1" s="266"/>
+      <c r="J1" s="266"/>
+      <c r="K1" s="266"/>
+      <c r="L1" s="266"/>
+      <c r="M1" s="266"/>
+      <c r="N1" s="266"/>
+      <c r="O1" s="266"/>
+      <c r="P1" s="266"/>
+      <c r="Q1" s="266"/>
+      <c r="R1" s="266"/>
+      <c r="S1" s="266"/>
+      <c r="T1" s="266"/>
+      <c r="U1" s="266"/>
+      <c r="V1" s="266"/>
+      <c r="W1" s="266"/>
+      <c r="X1" s="266"/>
+      <c r="Y1" s="266"/>
+      <c r="Z1" s="266"/>
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.15">
-      <c r="A2" s="262" t="s">
+      <c r="A2" s="266" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="262"/>
-      <c r="C2" s="262"/>
-      <c r="D2" s="262"/>
-      <c r="E2" s="262"/>
-      <c r="F2" s="262"/>
-      <c r="G2" s="262"/>
-      <c r="H2" s="262"/>
-      <c r="I2" s="262"/>
-      <c r="J2" s="262"/>
-      <c r="K2" s="262"/>
-      <c r="L2" s="262"/>
-      <c r="M2" s="262"/>
-      <c r="N2" s="262"/>
-      <c r="O2" s="262"/>
-      <c r="P2" s="262"/>
-      <c r="Q2" s="262"/>
-      <c r="R2" s="262"/>
-      <c r="S2" s="262"/>
-      <c r="T2" s="262"/>
-      <c r="U2" s="262"/>
-      <c r="V2" s="262"/>
-      <c r="W2" s="262"/>
-      <c r="X2" s="262"/>
-      <c r="Y2" s="262"/>
-      <c r="Z2" s="262"/>
+      <c r="B2" s="266"/>
+      <c r="C2" s="266"/>
+      <c r="D2" s="266"/>
+      <c r="E2" s="266"/>
+      <c r="F2" s="266"/>
+      <c r="G2" s="266"/>
+      <c r="H2" s="266"/>
+      <c r="I2" s="266"/>
+      <c r="J2" s="266"/>
+      <c r="K2" s="266"/>
+      <c r="L2" s="266"/>
+      <c r="M2" s="266"/>
+      <c r="N2" s="266"/>
+      <c r="O2" s="266"/>
+      <c r="P2" s="266"/>
+      <c r="Q2" s="266"/>
+      <c r="R2" s="266"/>
+      <c r="S2" s="266"/>
+      <c r="T2" s="266"/>
+      <c r="U2" s="266"/>
+      <c r="V2" s="266"/>
+      <c r="W2" s="266"/>
+      <c r="X2" s="266"/>
+      <c r="Y2" s="266"/>
+      <c r="Z2" s="266"/>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.15">
       <c r="C3" s="119" t="s">
@@ -17319,25 +17319,25 @@
     </row>
     <row r="4" spans="1:32" ht="14" thickBot="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:32" ht="14" thickTop="1" x14ac:dyDescent="0.15">
-      <c r="C5" s="263" t="s">
+      <c r="C5" s="267" t="s">
         <v>119</v>
       </c>
-      <c r="D5" s="263"/>
-      <c r="E5" s="263"/>
-      <c r="F5" s="263"/>
-      <c r="G5" s="263"/>
-      <c r="AC5" s="264" t="s">
+      <c r="D5" s="267"/>
+      <c r="E5" s="267"/>
+      <c r="F5" s="267"/>
+      <c r="G5" s="267"/>
+      <c r="AC5" s="268" t="s">
         <v>161</v>
       </c>
-      <c r="AD5" s="265"/>
+      <c r="AD5" s="269"/>
       <c r="AE5" s="119"/>
       <c r="AF5" s="119"/>
     </row>
     <row r="6" spans="1:32" ht="15" x14ac:dyDescent="0.15">
-      <c r="C6" s="266" t="s">
+      <c r="C6" s="270" t="s">
         <v>127</v>
       </c>
-      <c r="D6" s="266"/>
+      <c r="D6" s="270"/>
       <c r="E6" s="166" t="s">
         <v>177</v>
       </c>
@@ -17706,10 +17706,10 @@
       </c>
       <c r="D21" s="261"/>
       <c r="E21" s="261"/>
-      <c r="T21" s="267" t="s">
+      <c r="T21" s="262" t="s">
         <v>163</v>
       </c>
-      <c r="U21" s="268"/>
+      <c r="U21" s="263"/>
       <c r="V21" s="167" t="s">
         <v>154</v>
       </c>
@@ -17718,17 +17718,17 @@
       </c>
       <c r="X21" s="128"/>
       <c r="Y21" s="128"/>
-      <c r="Z21" s="269" t="s">
+      <c r="Z21" s="264" t="s">
         <v>157</v>
       </c>
-      <c r="AA21" s="269"/>
-      <c r="AB21" s="269"/>
+      <c r="AA21" s="264"/>
+      <c r="AB21" s="264"/>
     </row>
     <row r="22" spans="1:34" ht="15" x14ac:dyDescent="0.15">
-      <c r="A22" s="267" t="s">
+      <c r="A22" s="262" t="s">
         <v>153</v>
       </c>
-      <c r="B22" s="268"/>
+      <c r="B22" s="263"/>
       <c r="C22" s="133" t="s">
         <v>8</v>
       </c>
@@ -17780,10 +17780,10 @@
       <c r="S22" s="168" t="s">
         <v>176</v>
       </c>
-      <c r="T22" s="267" t="s">
+      <c r="T22" s="262" t="s">
         <v>188</v>
       </c>
-      <c r="U22" s="270"/>
+      <c r="U22" s="265"/>
       <c r="V22" s="168" t="s">
         <v>182</v>
       </c>
@@ -18492,17 +18492,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="T21:U21"/>
-    <mergeCell ref="Z21:AB21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="T22:U22"/>
     <mergeCell ref="T20:AB20"/>
     <mergeCell ref="A1:Z1"/>
     <mergeCell ref="A2:Z2"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="AC5:AD5"/>
     <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="T21:U21"/>
+    <mergeCell ref="Z21:AB21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="T22:U22"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X13 T32 T25:T28" xr:uid="{A3DEBC13-46CE-4D1E-BD8D-45F2ED5DBE94}">
@@ -18552,54 +18552,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.15">
-      <c r="A1" s="262" t="s">
+      <c r="A1" s="266" t="s">
         <v>151</v>
       </c>
-      <c r="B1" s="262"/>
-      <c r="C1" s="262"/>
-      <c r="D1" s="262"/>
-      <c r="E1" s="262"/>
-      <c r="F1" s="262"/>
-      <c r="G1" s="262"/>
-      <c r="H1" s="262"/>
-      <c r="I1" s="262"/>
-      <c r="J1" s="262"/>
-      <c r="K1" s="262"/>
-      <c r="L1" s="262"/>
-      <c r="M1" s="262"/>
-      <c r="N1" s="262"/>
-      <c r="O1" s="262"/>
-      <c r="P1" s="262"/>
-      <c r="Q1" s="262"/>
-      <c r="R1" s="262"/>
-      <c r="S1" s="262"/>
-      <c r="T1" s="262"/>
-      <c r="U1" s="262"/>
+      <c r="B1" s="266"/>
+      <c r="C1" s="266"/>
+      <c r="D1" s="266"/>
+      <c r="E1" s="266"/>
+      <c r="F1" s="266"/>
+      <c r="G1" s="266"/>
+      <c r="H1" s="266"/>
+      <c r="I1" s="266"/>
+      <c r="J1" s="266"/>
+      <c r="K1" s="266"/>
+      <c r="L1" s="266"/>
+      <c r="M1" s="266"/>
+      <c r="N1" s="266"/>
+      <c r="O1" s="266"/>
+      <c r="P1" s="266"/>
+      <c r="Q1" s="266"/>
+      <c r="R1" s="266"/>
+      <c r="S1" s="266"/>
+      <c r="T1" s="266"/>
+      <c r="U1" s="266"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.15">
-      <c r="A2" s="262" t="s">
+      <c r="A2" s="266" t="s">
         <v>150</v>
       </c>
-      <c r="B2" s="262"/>
-      <c r="C2" s="262"/>
-      <c r="D2" s="262"/>
-      <c r="E2" s="262"/>
-      <c r="F2" s="262"/>
-      <c r="G2" s="262"/>
-      <c r="H2" s="262"/>
-      <c r="I2" s="262"/>
-      <c r="J2" s="262"/>
-      <c r="K2" s="262"/>
-      <c r="L2" s="262"/>
-      <c r="M2" s="262"/>
-      <c r="N2" s="262"/>
-      <c r="O2" s="262"/>
-      <c r="P2" s="262"/>
-      <c r="Q2" s="262"/>
-      <c r="R2" s="262"/>
-      <c r="S2" s="262"/>
-      <c r="T2" s="262"/>
-      <c r="U2" s="262"/>
+      <c r="B2" s="266"/>
+      <c r="C2" s="266"/>
+      <c r="D2" s="266"/>
+      <c r="E2" s="266"/>
+      <c r="F2" s="266"/>
+      <c r="G2" s="266"/>
+      <c r="H2" s="266"/>
+      <c r="I2" s="266"/>
+      <c r="J2" s="266"/>
+      <c r="K2" s="266"/>
+      <c r="L2" s="266"/>
+      <c r="M2" s="266"/>
+      <c r="N2" s="266"/>
+      <c r="O2" s="266"/>
+      <c r="P2" s="266"/>
+      <c r="Q2" s="266"/>
+      <c r="R2" s="266"/>
+      <c r="S2" s="266"/>
+      <c r="T2" s="266"/>
+      <c r="U2" s="266"/>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.15">
       <c r="C3" s="119" t="s">
@@ -18609,25 +18609,25 @@
     </row>
     <row r="4" spans="1:27" ht="14" thickBot="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:27" ht="14" thickTop="1" x14ac:dyDescent="0.15">
-      <c r="C5" s="263" t="s">
+      <c r="C5" s="267" t="s">
         <v>119</v>
       </c>
-      <c r="D5" s="263"/>
-      <c r="E5" s="263"/>
-      <c r="F5" s="263"/>
-      <c r="G5" s="263"/>
-      <c r="X5" s="264" t="s">
+      <c r="D5" s="267"/>
+      <c r="E5" s="267"/>
+      <c r="F5" s="267"/>
+      <c r="G5" s="267"/>
+      <c r="X5" s="268" t="s">
         <v>161</v>
       </c>
-      <c r="Y5" s="265"/>
+      <c r="Y5" s="269"/>
       <c r="Z5" s="119"/>
       <c r="AA5" s="119"/>
     </row>
     <row r="6" spans="1:27" ht="15" x14ac:dyDescent="0.15">
-      <c r="C6" s="266" t="s">
+      <c r="C6" s="270" t="s">
         <v>127</v>
       </c>
-      <c r="D6" s="266"/>
+      <c r="D6" s="270"/>
       <c r="E6" s="166" t="s">
         <v>177</v>
       </c>
@@ -18953,10 +18953,10 @@
       </c>
       <c r="D21" s="261"/>
       <c r="E21" s="261"/>
-      <c r="O21" s="267" t="s">
+      <c r="O21" s="262" t="s">
         <v>163</v>
       </c>
-      <c r="P21" s="268"/>
+      <c r="P21" s="263"/>
       <c r="Q21" s="167" t="s">
         <v>154</v>
       </c>
@@ -18965,17 +18965,17 @@
       </c>
       <c r="S21" s="128"/>
       <c r="T21" s="128"/>
-      <c r="U21" s="269" t="s">
+      <c r="U21" s="264" t="s">
         <v>157</v>
       </c>
-      <c r="V21" s="269"/>
-      <c r="W21" s="269"/>
+      <c r="V21" s="264"/>
+      <c r="W21" s="264"/>
     </row>
     <row r="22" spans="1:23" ht="15" x14ac:dyDescent="0.15">
-      <c r="A22" s="267" t="s">
+      <c r="A22" s="262" t="s">
         <v>153</v>
       </c>
-      <c r="B22" s="268"/>
+      <c r="B22" s="263"/>
       <c r="C22" s="133" t="s">
         <v>8</v>
       </c>
@@ -19012,10 +19012,10 @@
       <c r="N22" s="168" t="s">
         <v>176</v>
       </c>
-      <c r="O22" s="267" t="s">
+      <c r="O22" s="262" t="s">
         <v>188</v>
       </c>
-      <c r="P22" s="270"/>
+      <c r="P22" s="265"/>
       <c r="Q22" s="168" t="s">
         <v>182</v>
       </c>
@@ -21547,29 +21547,29 @@
         <v>348.87361937825227</v>
       </c>
       <c r="H60" s="109">
-        <v>67.400000000000006</v>
+        <v>67.7</v>
       </c>
       <c r="I60" s="109">
-        <v>117.5</v>
+        <v>117.4</v>
       </c>
       <c r="J60" s="109">
-        <v>54.8</v>
+        <v>36.9</v>
       </c>
       <c r="K60" s="139">
         <f t="shared" ref="K60" si="30">Coef_1*G60*C60^4*H60^2/E60^2/10^9</f>
-        <v>6.1275443748904177</v>
+        <v>6.1822136450068887</v>
       </c>
       <c r="L60" s="138">
         <f t="shared" ref="L60" si="31">Coef_1*G60*D60^4*I60^2/E60^2/10^9</f>
-        <v>0.45571916558324194</v>
+        <v>0.45494380346829039</v>
       </c>
       <c r="M60" s="140">
         <f t="shared" ref="M60" si="32">K60/L60</f>
-        <v>13.445878158422891</v>
+        <v>13.588961093384338</v>
       </c>
       <c r="N60" s="138">
         <f t="shared" ref="N60" si="33">(3*(1/(PI()/2)^2)*G60*C60^2*D60^2*J60^2/E60^2)/10^9</f>
-        <v>0.81834079619638811</v>
+        <v>0.37104434556614768</v>
       </c>
       <c r="O60" s="121" t="s">
         <v>146</v>
@@ -21590,11 +21590,11 @@
       </c>
       <c r="T60" s="142">
         <f t="shared" ref="T60" si="35">(K60+(Q60/R60)^4*L60+(Q60/R60)^2*(Coef_3*K60+Coef_4*N60))*10^9</f>
-        <v>8986324784.4693947</v>
+        <v>8250709866.9683714</v>
       </c>
       <c r="U60" s="158">
         <f t="shared" ref="U60" si="36">S60/T60^0.5*1000</f>
-        <v>2.72429843832326</v>
+        <v>2.8431520039230516</v>
       </c>
     </row>
     <row r="66" spans="9:15" x14ac:dyDescent="0.15">
@@ -21632,17 +21632,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="U21:W21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="O22:P22"/>
     <mergeCell ref="O20:W20"/>
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="A2:U2"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="X5:Y5"/>
     <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="U21:W21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="O22:P22"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S13 O25:O34 O36:O37 O40:O47 O50:O57 O60" xr:uid="{664F27CC-03B8-41DD-9E77-6535CBE6D30A}">

</xml_diff>